<commit_message>
Actualizacion automatica Informe Semanal DEX
</commit_message>
<xml_diff>
--- a/links/links_dex.xlsx
+++ b/links/links_dex.xlsx
@@ -469,12 +469,12 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>https://OperacionesAdecco.github.io/InformesRutas_DEX/dex/atipana-dex-s-a-c.html</t>
+          <t>https://OperacionesAdecco.github.io/Consolidado_InformesDEX/dex/atipana-dex-s-a-c.html</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>https://OperacionesAdecco.github.io/InformesRutas_DEX/capturas/atipana-dex-s-a-c.png</t>
+          <t>https://OperacionesAdecco.github.io/Consolidado_InformesDEX/capturas/atipana-dex-s-a-c.png</t>
         </is>
       </c>
     </row>
@@ -486,12 +486,12 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>https://OperacionesAdecco.github.io/InformesRutas_DEX/dex/atuq-dex-s-a-c.html</t>
+          <t>https://OperacionesAdecco.github.io/Consolidado_InformesDEX/dex/atuq-dex-s-a-c.html</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>https://OperacionesAdecco.github.io/InformesRutas_DEX/capturas/atuq-dex-s-a-c.png</t>
+          <t>https://OperacionesAdecco.github.io/Consolidado_InformesDEX/capturas/atuq-dex-s-a-c.png</t>
         </is>
       </c>
     </row>
@@ -503,12 +503,12 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>https://OperacionesAdecco.github.io/InformesRutas_DEX/dex/d-l-f-medina-rivera-s-a.html</t>
+          <t>https://OperacionesAdecco.github.io/Consolidado_InformesDEX/dex/d-l-f-medina-rivera-s-a.html</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>https://OperacionesAdecco.github.io/InformesRutas_DEX/capturas/d-l-f-medina-rivera-s-a.png</t>
+          <t>https://OperacionesAdecco.github.io/Consolidado_InformesDEX/capturas/d-l-f-medina-rivera-s-a.png</t>
         </is>
       </c>
     </row>
@@ -520,12 +520,12 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>https://OperacionesAdecco.github.io/InformesRutas_DEX/dex/distribuidora-aurelio-s-a-c.html</t>
+          <t>https://OperacionesAdecco.github.io/Consolidado_InformesDEX/dex/distribuidora-aurelio-s-a-c.html</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>https://OperacionesAdecco.github.io/InformesRutas_DEX/capturas/distribuidora-aurelio-s-a-c.png</t>
+          <t>https://OperacionesAdecco.github.io/Consolidado_InformesDEX/capturas/distribuidora-aurelio-s-a-c.png</t>
         </is>
       </c>
     </row>
@@ -537,12 +537,12 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>https://OperacionesAdecco.github.io/InformesRutas_DEX/dex/distribuidora-cunza-s-a.html</t>
+          <t>https://OperacionesAdecco.github.io/Consolidado_InformesDEX/dex/distribuidora-cunza-s-a.html</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>https://OperacionesAdecco.github.io/InformesRutas_DEX/capturas/distribuidora-cunza-s-a.png</t>
+          <t>https://OperacionesAdecco.github.io/Consolidado_InformesDEX/capturas/distribuidora-cunza-s-a.png</t>
         </is>
       </c>
     </row>
@@ -554,12 +554,12 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>https://OperacionesAdecco.github.io/InformesRutas_DEX/dex/distribuidora-sol-del-valle-s-a-c.html</t>
+          <t>https://OperacionesAdecco.github.io/Consolidado_InformesDEX/dex/distribuidora-sol-del-valle-s-a-c.html</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>https://OperacionesAdecco.github.io/InformesRutas_DEX/capturas/distribuidora-sol-del-valle-s-a-c.png</t>
+          <t>https://OperacionesAdecco.github.io/Consolidado_InformesDEX/capturas/distribuidora-sol-del-valle-s-a-c.png</t>
         </is>
       </c>
     </row>
@@ -571,12 +571,12 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>https://OperacionesAdecco.github.io/InformesRutas_DEX/dex/fuerzadex-s-a-c.html</t>
+          <t>https://OperacionesAdecco.github.io/Consolidado_InformesDEX/dex/fuerzadex-s-a-c.html</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>https://OperacionesAdecco.github.io/InformesRutas_DEX/capturas/fuerzadex-s-a-c.png</t>
+          <t>https://OperacionesAdecco.github.io/Consolidado_InformesDEX/capturas/fuerzadex-s-a-c.png</t>
         </is>
       </c>
     </row>
@@ -588,12 +588,12 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>https://OperacionesAdecco.github.io/InformesRutas_DEX/dex/pacifico-ayacucho.html</t>
+          <t>https://OperacionesAdecco.github.io/Consolidado_InformesDEX/dex/pacifico-ayacucho.html</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>https://OperacionesAdecco.github.io/InformesRutas_DEX/capturas/pacifico-ayacucho.png</t>
+          <t>https://OperacionesAdecco.github.io/Consolidado_InformesDEX/capturas/pacifico-ayacucho.png</t>
         </is>
       </c>
     </row>
@@ -605,12 +605,12 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>https://OperacionesAdecco.github.io/InformesRutas_DEX/dex/pacifico-dex-sociedad-anonima-cerrada.html</t>
+          <t>https://OperacionesAdecco.github.io/Consolidado_InformesDEX/dex/pacifico-dex-sociedad-anonima-cerrada.html</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>https://OperacionesAdecco.github.io/InformesRutas_DEX/capturas/pacifico-dex-sociedad-anonima-cerrada.png</t>
+          <t>https://OperacionesAdecco.github.io/Consolidado_InformesDEX/capturas/pacifico-dex-sociedad-anonima-cerrada.png</t>
         </is>
       </c>
     </row>
@@ -622,12 +622,12 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>https://OperacionesAdecco.github.io/InformesRutas_DEX/dex/pardadex.html</t>
+          <t>https://OperacionesAdecco.github.io/Consolidado_InformesDEX/dex/pardadex.html</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>https://OperacionesAdecco.github.io/InformesRutas_DEX/capturas/pardadex.png</t>
+          <t>https://OperacionesAdecco.github.io/Consolidado_InformesDEX/capturas/pardadex.png</t>
         </is>
       </c>
     </row>
@@ -639,12 +639,12 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>https://OperacionesAdecco.github.io/InformesRutas_DEX/dex/roset-distribuciones-eirl.html</t>
+          <t>https://OperacionesAdecco.github.io/Consolidado_InformesDEX/dex/roset-distribuciones-eirl.html</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>https://OperacionesAdecco.github.io/InformesRutas_DEX/capturas/roset-distribuciones-eirl.png</t>
+          <t>https://OperacionesAdecco.github.io/Consolidado_InformesDEX/capturas/roset-distribuciones-eirl.png</t>
         </is>
       </c>
     </row>

</xml_diff>